<commit_message>
Verificação de aderência de processo refeita
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/FS - Checklist Verificacao de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/FS - Checklist Verificacao de Projeto.xlsx
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="122">
   <si>
     <t>IAP - Indicador de Aderência ao Processo (70% a 100%)</t>
   </si>
@@ -312,7 +312,7 @@
     <t>Existe template para documento não previsto no SpinOff?</t>
   </si>
   <si>
-    <t>Não</t>
+    <t>NA</t>
   </si>
   <si>
     <t>Todos os templates e arquivos presentes são previstos no SpinOff</t>
@@ -348,10 +348,10 @@
     <t>Caso tenha sido criado o protótipo, ele foi armazenado na pasta correta da estrutura do projeto?</t>
   </si>
   <si>
-    <t>NA</t>
+    <t>O escopo foi apresentado e aprovado pelo cliente ou representante?</t>
   </si>
   <si>
-    <t>O escopo foi apresentado e aprovado pelo cliente ou representante?</t>
+    <t>Não</t>
   </si>
   <si>
     <t>O escopo foi reformulado e a nova versão ainda não foi apresentada ao cliente</t>
@@ -409,6 +409,9 @@
   </si>
   <si>
     <t>Os históricos de atualizações dos artefatos, na ferramenta,  possuem descrição do que foi alterado?</t>
+  </si>
+  <si>
+    <t>Os artefatos não sofreram atualizações até o momento</t>
   </si>
   <si>
     <t>O visão foi atualizado devido a mudança de escopo?</t>
@@ -1048,11 +1051,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="172840240"/>
-        <c:axId val="1835878332"/>
+        <c:axId val="1080490920"/>
+        <c:axId val="426640699"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="172840240"/>
+        <c:axId val="1080490920"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1104,10 +1107,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1835878332"/>
+        <c:crossAx val="426640699"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1835878332"/>
+        <c:axId val="426640699"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1171,7 +1174,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="172840240"/>
+        <c:crossAx val="1080490920"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1326,11 +1329,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1037977287"/>
-        <c:axId val="1963265887"/>
+        <c:axId val="636362806"/>
+        <c:axId val="545702460"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1037977287"/>
+        <c:axId val="636362806"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1382,10 +1385,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1963265887"/>
+        <c:crossAx val="545702460"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1963265887"/>
+        <c:axId val="545702460"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1449,7 +1452,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1037977287"/>
+        <c:crossAx val="636362806"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1590,11 +1593,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="91385342"/>
-        <c:axId val="137790198"/>
+        <c:axId val="926936422"/>
+        <c:axId val="975831747"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91385342"/>
+        <c:axId val="926936422"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1646,10 +1649,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="137790198"/>
+        <c:crossAx val="975831747"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="137790198"/>
+        <c:axId val="975831747"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1661,7 +1664,7 @@
             <a:noFill/>
           </a:ln>
         </c:spPr>
-        <c:crossAx val="91385342"/>
+        <c:crossAx val="926936422"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1802,11 +1805,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="320757239"/>
-        <c:axId val="1808496276"/>
+        <c:axId val="541344789"/>
+        <c:axId val="1378598527"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="320757239"/>
+        <c:axId val="541344789"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1858,10 +1861,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1808496276"/>
+        <c:crossAx val="1378598527"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1808496276"/>
+        <c:axId val="1378598527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1873,7 +1876,7 @@
             <a:noFill/>
           </a:ln>
         </c:spPr>
-        <c:crossAx val="320757239"/>
+        <c:crossAx val="541344789"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2014,11 +2017,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="821524621"/>
-        <c:axId val="46235794"/>
+        <c:axId val="1575361722"/>
+        <c:axId val="472691564"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="821524621"/>
+        <c:axId val="1575361722"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2070,10 +2073,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46235794"/>
+        <c:crossAx val="472691564"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46235794"/>
+        <c:axId val="472691564"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2085,7 +2088,7 @@
             <a:noFill/>
           </a:ln>
         </c:spPr>
-        <c:crossAx val="821524621"/>
+        <c:crossAx val="1575361722"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2492,7 +2495,7 @@
       </c>
       <c r="B3" s="5">
         <f>'Ver-Iniciação1'!$F$2</f>
-        <v>0.8636363636</v>
+        <v>0.8571428571</v>
       </c>
     </row>
     <row r="4">
@@ -5578,11 +5581,11 @@
       </c>
       <c r="D2" s="8">
         <f>('Ver-Iniciação1'!$I$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="8">
         <f>('Ver-Iniciação1'!$J$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" s="7" t="s">
         <v>13</v>
@@ -5930,7 +5933,7 @@
       </c>
       <c r="B11" s="8">
         <f>('Ver-Iniciação1'!$G$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="C11" s="8">
         <f>('Ver-Iniciação1'!$H$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
@@ -5938,7 +5941,7 @@
       </c>
       <c r="D11" s="8">
         <f>('Ver-Iniciação1'!$I$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E11" s="8">
         <f>('Ver-Iniciação1'!$J$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
@@ -7520,7 +7523,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.14"/>
+    <col customWidth="1" min="1" max="1" width="46.57"/>
     <col customWidth="1" min="2" max="2" width="5.29"/>
     <col customWidth="1" min="3" max="3" width="84.0"/>
     <col customWidth="1" min="4" max="4" width="9.86"/>
@@ -7557,7 +7560,7 @@
       <c r="E2" s="15"/>
       <c r="F2" s="16">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
-        <v>0.8636363636</v>
+        <v>0.8571428571</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1">
@@ -7615,11 +7618,11 @@
       </c>
       <c r="I5" s="7">
         <f>COUNTIF(D6,"Não")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="7">
         <f>COUNTIF(D6,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="18.75" customHeight="1">
@@ -7873,7 +7876,7 @@
         <v>54</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E17" s="30"/>
       <c r="F17" s="30"/>
@@ -7904,10 +7907,10 @@
         <v>11.0</v>
       </c>
       <c r="C18" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="31" t="s">
         <v>56</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>43</v>
       </c>
       <c r="E18" s="32" t="s">
         <v>57</v>
@@ -7969,7 +7972,7 @@
         <v>59</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E20" s="30"/>
       <c r="F20" s="30"/>
@@ -7983,7 +7986,7 @@
         <v>60</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E21" s="30"/>
       <c r="F21" s="30"/>
@@ -8023,7 +8026,7 @@
         <v>46</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E23" s="30"/>
       <c r="F23" s="30"/>
@@ -8037,7 +8040,7 @@
         <v>61</v>
       </c>
       <c r="D24" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E24" s="30"/>
       <c r="F24" s="30"/>
@@ -8077,7 +8080,7 @@
         <v>46</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E26" s="30"/>
       <c r="F26" s="30"/>
@@ -8091,7 +8094,7 @@
         <v>62</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E27" s="30"/>
       <c r="F27" s="30"/>
@@ -8205,7 +8208,7 @@
       </c>
       <c r="F34" s="30"/>
     </row>
-    <row r="35" ht="18.75" customHeight="1">
+    <row r="35">
       <c r="A35" s="33"/>
       <c r="B35" s="29">
         <v>27.0</v>
@@ -8228,7 +8231,7 @@
         <v>69</v>
       </c>
       <c r="D36" s="32" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="E36" s="32" t="s">
         <v>70</v>
@@ -8248,7 +8251,7 @@
       <c r="F37" s="27"/>
       <c r="G37" s="7">
         <f>COUNTIF(D38:D41,"Sim")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H37" s="7">
         <f>COUNTIF(D38:D41,"Parcialmente")</f>
@@ -8256,7 +8259,7 @@
       </c>
       <c r="I37" s="7">
         <f>COUNTIF(D38:D41,"Não")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="7">
         <f>COUNTIF(D38:D41,"NA")</f>
@@ -8305,7 +8308,7 @@
       <c r="E40" s="30"/>
       <c r="F40" s="30"/>
     </row>
-    <row r="41" ht="20.25" customHeight="1">
+    <row r="41">
       <c r="A41" s="42"/>
       <c r="B41" s="29">
         <v>33.0</v>
@@ -8314,9 +8317,11 @@
         <v>75</v>
       </c>
       <c r="D41" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="30"/>
+        <v>56</v>
+      </c>
+      <c r="E41" s="32" t="s">
+        <v>76</v>
+      </c>
       <c r="F41" s="30"/>
     </row>
     <row r="42" ht="18.75" customHeight="1">
@@ -12272,7 +12277,7 @@
         <v>1.0</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" s="48"/>
       <c r="E6" s="30"/>
@@ -12310,7 +12315,7 @@
         <v>2.0</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="48"/>
       <c r="E8" s="30"/>
@@ -12354,7 +12359,7 @@
         <v>3.0</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="48"/>
       <c r="E9" s="30"/>
@@ -12392,7 +12397,7 @@
         <v>4.0</v>
       </c>
       <c r="C11" s="35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D11" s="48"/>
       <c r="E11" s="30"/>
@@ -12420,7 +12425,7 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12" s="48"/>
       <c r="E12" s="30"/>
@@ -12432,7 +12437,7 @@
         <v>6.0</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D13" s="48"/>
       <c r="E13" s="30"/>
@@ -12444,7 +12449,7 @@
         <v>7.0</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D14" s="48"/>
       <c r="E14" s="30"/>
@@ -12466,7 +12471,7 @@
         <v>7.0</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" s="48"/>
       <c r="E16" s="30"/>
@@ -12490,7 +12495,7 @@
     </row>
     <row r="17" ht="15.0" customHeight="1">
       <c r="A17" s="24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B17" s="25"/>
       <c r="C17" s="26" t="s">
@@ -12506,7 +12511,7 @@
         <v>9.0</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D18" s="48"/>
       <c r="E18" s="30"/>
@@ -12534,7 +12539,7 @@
         <v>10.0</v>
       </c>
       <c r="C19" s="35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D19" s="48"/>
       <c r="E19" s="30"/>
@@ -12546,7 +12551,7 @@
         <v>11.0</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D20" s="48"/>
       <c r="E20" s="30"/>
@@ -12578,7 +12583,7 @@
         <v>12.0</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D21" s="48"/>
       <c r="E21" s="30"/>
@@ -12586,7 +12591,7 @@
     </row>
     <row r="22" ht="18.75" customHeight="1">
       <c r="A22" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" s="25"/>
       <c r="C22" s="26" t="s">
@@ -12602,7 +12607,7 @@
         <v>17.0</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D23" s="48"/>
       <c r="E23" s="30"/>
@@ -12630,7 +12635,7 @@
         <v>18.0</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D24" s="48"/>
       <c r="E24" s="30"/>
@@ -12642,7 +12647,7 @@
         <v>19.0</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D25" s="48"/>
       <c r="E25" s="30"/>
@@ -12654,7 +12659,7 @@
         <v>21.0</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D26" s="48"/>
       <c r="E26" s="30"/>
@@ -12666,7 +12671,7 @@
         <v>22.0</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D27" s="48"/>
       <c r="E27" s="30"/>
@@ -12674,7 +12679,7 @@
     </row>
     <row r="28" ht="18.75" customHeight="1">
       <c r="A28" s="24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B28" s="25"/>
       <c r="C28" s="26" t="s">
@@ -12690,7 +12695,7 @@
         <v>23.0</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D29" s="48"/>
       <c r="E29" s="30"/>
@@ -12718,7 +12723,7 @@
         <v>24.0</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D30" s="48"/>
       <c r="E30" s="30"/>
@@ -12730,7 +12735,7 @@
         <v>25.0</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D31" s="48"/>
       <c r="E31" s="30"/>
@@ -12742,7 +12747,7 @@
         <v>26.0</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D32" s="48"/>
       <c r="E32" s="30"/>
@@ -12754,7 +12759,7 @@
         <v>27.0</v>
       </c>
       <c r="C33" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D33" s="48"/>
       <c r="E33" s="30"/>
@@ -12766,7 +12771,7 @@
         <v>28.0</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D34" s="48"/>
       <c r="E34" s="30"/>
@@ -12852,7 +12857,7 @@
         <v>32.0</v>
       </c>
       <c r="C40" s="30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D40" s="48"/>
       <c r="E40" s="30"/>
@@ -12880,7 +12885,7 @@
         <v>33.0</v>
       </c>
       <c r="C41" s="30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D41" s="48"/>
       <c r="E41" s="30"/>
@@ -16843,7 +16848,7 @@
         <v>1.0</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" s="48"/>
       <c r="E6" s="30"/>
@@ -16881,7 +16886,7 @@
         <v>2.0</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="48"/>
       <c r="E8" s="30"/>
@@ -16935,7 +16940,7 @@
         <v>3.0</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" s="48"/>
       <c r="E10" s="30"/>
@@ -16963,7 +16968,7 @@
         <v>4.0</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" s="48"/>
       <c r="E11" s="30"/>
@@ -16975,7 +16980,7 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D12" s="48"/>
       <c r="E12" s="30"/>
@@ -16997,7 +17002,7 @@
         <v>6.0</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" s="48"/>
       <c r="E14" s="30"/>
@@ -17021,7 +17026,7 @@
     </row>
     <row r="15" ht="15.0" customHeight="1">
       <c r="A15" s="24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="26" t="s">
@@ -17037,7 +17042,7 @@
         <v>8.0</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D16" s="48"/>
       <c r="E16" s="30"/>
@@ -17061,7 +17066,7 @@
     </row>
     <row r="17" ht="18.75" customHeight="1">
       <c r="A17" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B17" s="25"/>
       <c r="C17" s="26" t="s">
@@ -17077,7 +17082,7 @@
         <v>11.0</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D18" s="48"/>
       <c r="E18" s="30"/>
@@ -17105,7 +17110,7 @@
         <v>13.0</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D19" s="48"/>
       <c r="E19" s="30"/>
@@ -17117,7 +17122,7 @@
         <v>14.0</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D20" s="48"/>
       <c r="E20" s="30"/>
@@ -17129,7 +17134,7 @@
         <v>15.0</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D21" s="48"/>
       <c r="E21" s="30"/>
@@ -17141,7 +17146,7 @@
         <v>16.0</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D22" s="48"/>
       <c r="E22" s="30"/>
@@ -17149,7 +17154,7 @@
     </row>
     <row r="23" ht="18.75" customHeight="1">
       <c r="A23" s="24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="26" t="s">
@@ -17193,7 +17198,7 @@
         <v>18.0</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D25" s="48"/>
       <c r="E25" s="30"/>
@@ -17205,7 +17210,7 @@
         <v>19.0</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D26" s="48"/>
       <c r="E26" s="30"/>
@@ -17217,7 +17222,7 @@
         <v>21.0</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D27" s="48"/>
       <c r="E27" s="30"/>
@@ -17229,7 +17234,7 @@
         <v>22.0</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D28" s="48"/>
       <c r="E28" s="30"/>
@@ -17237,7 +17242,7 @@
     </row>
     <row r="29" ht="18.75" customHeight="1">
       <c r="A29" s="24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B29" s="25"/>
       <c r="C29" s="26" t="s">
@@ -17253,7 +17258,7 @@
         <v>24.0</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D30" s="48"/>
       <c r="E30" s="30"/>
@@ -17281,7 +17286,7 @@
         <v>26.0</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D31" s="48"/>
       <c r="E31" s="30"/>
@@ -17293,7 +17298,7 @@
         <v>27.0</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D32" s="48"/>
       <c r="E32" s="30"/>
@@ -17305,7 +17310,7 @@
         <v>28.0</v>
       </c>
       <c r="C33" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D33" s="48"/>
       <c r="E33" s="30"/>
@@ -17317,7 +17322,7 @@
         <v>29.0</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D34" s="48"/>
       <c r="E34" s="30"/>
@@ -17391,7 +17396,7 @@
       <c r="A39" s="41"/>
       <c r="B39" s="29"/>
       <c r="C39" s="30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D39" s="48"/>
       <c r="E39" s="30"/>
@@ -17413,7 +17418,7 @@
         <v>33.0</v>
       </c>
       <c r="C41" s="30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D41" s="48"/>
       <c r="E41" s="30"/>
@@ -17441,7 +17446,7 @@
         <v>34.0</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D42" s="48"/>
       <c r="E42" s="30"/>
@@ -21380,7 +21385,7 @@
         <v>1.0</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" s="48"/>
       <c r="E6" s="30"/>
@@ -21418,7 +21423,7 @@
         <v>2.0</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="48"/>
       <c r="E8" s="30"/>
@@ -21472,7 +21477,7 @@
         <v>3.0</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" s="48"/>
       <c r="E10" s="30"/>
@@ -21500,7 +21505,7 @@
         <v>4.0</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" s="48"/>
       <c r="E11" s="30"/>
@@ -21512,7 +21517,7 @@
         <v>5.0</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D12" s="48"/>
       <c r="E12" s="30"/>
@@ -21534,7 +21539,7 @@
         <v>6.0</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" s="48"/>
       <c r="E14" s="30"/>
@@ -21558,7 +21563,7 @@
     </row>
     <row r="15" ht="15.0" customHeight="1">
       <c r="A15" s="24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="26" t="s">
@@ -21574,7 +21579,7 @@
         <v>8.0</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D16" s="48"/>
       <c r="E16" s="30"/>
@@ -21598,7 +21603,7 @@
     </row>
     <row r="17" ht="15.0" customHeight="1">
       <c r="A17" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B17" s="25"/>
       <c r="C17" s="26" t="s">
@@ -21614,7 +21619,7 @@
         <v>9.0</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D18" s="48"/>
       <c r="E18" s="30"/>
@@ -21642,7 +21647,7 @@
         <v>10.0</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D19" s="48"/>
       <c r="E19" s="30"/>
@@ -21654,7 +21659,7 @@
         <v>11.0</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D20" s="48"/>
       <c r="E20" s="30"/>
@@ -21666,7 +21671,7 @@
         <v>13.0</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D21" s="48"/>
       <c r="E21" s="30"/>
@@ -21674,7 +21679,7 @@
     </row>
     <row r="22" ht="18.75" customHeight="1">
       <c r="A22" s="24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B22" s="25"/>
       <c r="C22" s="26" t="s">
@@ -21690,7 +21695,7 @@
         <v>14.0</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D23" s="48"/>
       <c r="E23" s="30"/>
@@ -21718,7 +21723,7 @@
         <v>15.0</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D24" s="48"/>
       <c r="E24" s="30"/>
@@ -21726,7 +21731,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B25" s="25"/>
       <c r="C25" s="26" t="s">
@@ -21806,7 +21811,7 @@
         <v>25.0</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D27" s="48"/>
       <c r="E27" s="30"/>
@@ -21872,7 +21877,7 @@
     </row>
     <row r="30" ht="18.75" customHeight="1">
       <c r="A30" s="24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B30" s="25"/>
       <c r="C30" s="26" t="s">
@@ -21888,7 +21893,7 @@
         <v>19.0</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D31" s="48"/>
       <c r="E31" s="30"/>
@@ -21916,7 +21921,7 @@
         <v>20.0</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D32" s="48"/>
       <c r="E32" s="30"/>
@@ -21928,7 +21933,7 @@
         <v>21.0</v>
       </c>
       <c r="C33" s="30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D33" s="48"/>
       <c r="E33" s="30"/>
@@ -21940,7 +21945,7 @@
         <v>24.0</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D34" s="48"/>
       <c r="E34" s="30"/>
@@ -21952,7 +21957,7 @@
         <v>25.0</v>
       </c>
       <c r="C35" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D35" s="48"/>
       <c r="E35" s="30"/>
@@ -22026,7 +22031,7 @@
       <c r="A40" s="41"/>
       <c r="B40" s="29"/>
       <c r="C40" s="30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D40" s="48"/>
       <c r="E40" s="30"/>
@@ -22048,7 +22053,7 @@
         <v>29.0</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D42" s="48"/>
       <c r="E42" s="30"/>
@@ -22076,7 +22081,7 @@
         <v>30.0</v>
       </c>
       <c r="C43" s="30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D43" s="48"/>
       <c r="E43" s="30"/>

</xml_diff>